<commit_message>
Fähigkeit statt Subkompetenz, Fachkommentar-Pflicht bei *, Skala im Template, Branding
- Spalte/Begriff "Subkompetenz" -> "Fähigkeit" (Template, Beispiel, UI, README)
- Validierung: wird in einem Fach "*" vergeben, muss der Fachkommentar
  (ein Feld pro Fach, erste Zeile) ausgefuellt sein
- Excel-Vorlage zeigt die Bewertungsskala (1-5, *) oben rechts (Spalten D/E)
- Branding: GKS-Logo + Titel "Zeugnis-Generator / Georg-Kerschensteiner-Schule"
  im Seitenkopf, Akzentlinie; <title> angepasst

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/zeugnis-vorlage.xlsx
+++ b/zeugnis-vorlage.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E108"/>
+  <dimension ref="A1:E112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -441,9 +441,17 @@
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
+      <c r="C1" s="2" t="inlineStr"/>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Bewertung</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Bedeutung</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -456,9 +464,17 @@
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>sicher</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -467,106 +483,126 @@
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>überwiegend</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>teilweise</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>Fach</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>Kompetenz</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t>Subkompetenz</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>Bewertung</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>Fachkommentar</t>
+      <c r="A5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>mit Unterstützung</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Deutsch</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Sprechen und Zuhören</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Du gibst Informationen korrekt wieder.</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>noch nicht erworben (→)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr"/>
       <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Du beziehst dich auf die Beiträge anderer.</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>siehe Kommentar</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Du kannst grammatikalisch richtige Sätze bilden.</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Lesen und Texte rezipieren</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Du kannst altersgemäße Texte in angemessener Zeit lesen und verstehen.</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Fach</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>Kompetenz</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>Fähigkeit</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Bewertung</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>Fachkommentar</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
-      <c r="B10" s="2" t="inlineStr"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Sprechen und Zuhören</t>
+        </is>
+      </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Fragen zum Gelesenen mündlich und schriftlich beantworten.</t>
+          <t>Du gibst Informationen korrekt wieder.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
@@ -577,7 +613,7 @@
       <c r="B11" s="2" t="inlineStr"/>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Du markierst wichtige Aussagen eines Textes passend.</t>
+          <t>Du beziehst dich auf die Beiträge anderer.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
@@ -588,7 +624,7 @@
       <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Du kannst den Inhalt des Gelesenen in Stichworten notieren.</t>
+          <t>Du kannst grammatikalisch richtige Sätze bilden.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
@@ -596,10 +632,14 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr"/>
-      <c r="B13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Lesen und Texte rezipieren</t>
+        </is>
+      </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Du kannst wichtige Inhalte des Gelesenen erfassen und mithilfe von Textstellen belegen.</t>
+          <t>Du kannst altersgemäße Texte in angemessener Zeit lesen und verstehen.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
@@ -610,7 +650,7 @@
       <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Du äußerst zu altersgemäßen Texten eigene Gedanken und Einschätzungen.</t>
+          <t>Du kannst Fragen zum Gelesenen mündlich und schriftlich beantworten.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
@@ -621,7 +661,7 @@
       <c r="B15" s="2" t="inlineStr"/>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Du kannst geübte Texte flüssig und mit Betonung vorlesen.</t>
+          <t>Du markierst wichtige Aussagen eines Textes passend.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
@@ -629,14 +669,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr"/>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Schreiben</t>
-        </is>
-      </c>
+      <c r="B16" s="2" t="inlineStr"/>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Du schreibst lesbar und zügig.</t>
+          <t>Du kannst den Inhalt des Gelesenen in Stichworten notieren.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
@@ -647,7 +683,7 @@
       <c r="B17" s="2" t="inlineStr"/>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Du wendest Rechtschreibstrategien auch bei unbekannten Wörtern richtig an.</t>
+          <t>Du kannst wichtige Inhalte des Gelesenen erfassen und mithilfe von Textstellen belegen.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
@@ -658,7 +694,7 @@
       <c r="B18" s="2" t="inlineStr"/>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Du schreibst geübte Wörter aus dem Grundwortschatz richtig.</t>
+          <t>Du äußerst zu altersgemäßen Texten eigene Gedanken und Einschätzungen.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
@@ -669,7 +705,7 @@
       <c r="B19" s="2" t="inlineStr"/>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Du schreibst Nomen und Satzanfänge groß.</t>
+          <t>Du kannst geübte Texte flüssig und mit Betonung vorlesen.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
@@ -677,10 +713,14 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr"/>
-      <c r="B20" s="2" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Schreiben</t>
+        </is>
+      </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Du hältst Wort- und Satzgrenzen ein.</t>
+          <t>Du schreibst lesbar und zügig.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
@@ -691,7 +731,7 @@
       <c r="B21" s="2" t="inlineStr"/>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Du gliederst deine Texte übersichtlich.</t>
+          <t>Du wendest Rechtschreibstrategien auch bei unbekannten Wörtern richtig an.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
@@ -702,7 +742,7 @@
       <c r="B22" s="2" t="inlineStr"/>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Du schreibst fehlerfrei ab.</t>
+          <t>Du schreibst geübte Wörter aus dem Grundwortschatz richtig.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
@@ -713,7 +753,7 @@
       <c r="B23" s="2" t="inlineStr"/>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Du kannst das Wörterbuch als Rechtschreibhilfe nutzen.</t>
+          <t>Du schreibst Nomen und Satzanfänge groß.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
@@ -724,7 +764,7 @@
       <c r="B24" s="2" t="inlineStr"/>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Du kannst vollständige, grammatikalisch richtige Sätze schreiben.</t>
+          <t>Du hältst Wort- und Satzgrenzen ein.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
@@ -735,7 +775,7 @@
       <c r="B25" s="2" t="inlineStr"/>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Du schreibst Geschichten, Berichte und Personenbeschreibungen nach besprochenen Kriterien.</t>
+          <t>Du gliederst deine Texte übersichtlich.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
@@ -746,7 +786,7 @@
       <c r="B26" s="2" t="inlineStr"/>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Du entwickelst Schreibideen für Texte.</t>
+          <t>Du schreibst fehlerfrei ab.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
@@ -757,7 +797,7 @@
       <c r="B27" s="2" t="inlineStr"/>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Du gestaltest eigene Texte mit Hilfe sprachlicher Mittel (z. B. wechselnde Satzanfänge, passende Zeitformen, wörtliche Rede).</t>
+          <t>Du kannst das Wörterbuch als Rechtschreibhilfe nutzen.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
@@ -768,7 +808,7 @@
       <c r="B28" s="2" t="inlineStr"/>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Du reflektierst und überarbeitest deine Texte.</t>
+          <t>Du kannst vollständige, grammatikalisch richtige Sätze schreiben.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr"/>
@@ -779,7 +819,7 @@
       <c r="B29" s="2" t="inlineStr"/>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Du präsentierst deine Texte vor anderen.</t>
+          <t>Du schreibst Geschichten, Berichte und Personenbeschreibungen nach besprochenen Kriterien.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr"/>
@@ -787,14 +827,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr"/>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Sprache untersuchen</t>
-        </is>
-      </c>
+      <c r="B30" s="2" t="inlineStr"/>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Du ordnest Wörter den Wortarten Nomen, Adjektive, Verben, Artikel, Präpositionen und Pronomen passend zu.</t>
+          <t>Du entwickelst Schreibideen für Texte.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr"/>
@@ -805,7 +841,7 @@
       <c r="B31" s="2" t="inlineStr"/>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Du unterscheidest Aussage-, Frage- und Ausrufesatz und verwendest die passenden Satzschlusszeichen.</t>
+          <t>Du gestaltest eigene Texte mit Hilfe sprachlicher Mittel (z. B. wechselnde Satzanfänge, passende Zeitformen, wörtliche Rede).</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr"/>
@@ -816,7 +852,7 @@
       <c r="B32" s="2" t="inlineStr"/>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Du erkennst die wörtliche Rede und setzt die passenden Satzzeichen.</t>
+          <t>Du reflektierst und überarbeitest deine Texte.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr"/>
@@ -827,7 +863,7 @@
       <c r="B33" s="2" t="inlineStr"/>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Du benennst und bildest Verbformen in verschiedenen Zeiten (Präsens, Präteritum, Perfekt) richtig.</t>
+          <t>Du präsentierst deine Texte vor anderen.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr"/>
@@ -835,29 +871,25 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr"/>
-      <c r="B34" s="2" t="inlineStr"/>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Sprache untersuchen</t>
+        </is>
+      </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Wörter nach dem Alphabet sortieren und nachschlagen.</t>
+          <t>Du ordnest Wörter den Wortarten Nomen, Adjektive, Verben, Artikel, Präpositionen und Pronomen passend zu.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Mathematik</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Zahl und Operation (Zahlenraum bis 1.000)</t>
-        </is>
-      </c>
+      <c r="A35" s="2" t="inlineStr"/>
+      <c r="B35" s="2" t="inlineStr"/>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Du kannst dich im Zahlenraum bis 1000 orientieren.</t>
+          <t>Du unterscheidest Aussage-, Frage- und Ausrufesatz und verwendest die passenden Satzschlusszeichen.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr"/>
@@ -868,7 +900,7 @@
       <c r="B36" s="2" t="inlineStr"/>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Additionsaufgaben (+) mit und ohne Übergänge lösen.</t>
+          <t>Du erkennst die wörtliche Rede und setzt die passenden Satzzeichen.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr"/>
@@ -879,7 +911,7 @@
       <c r="B37" s="2" t="inlineStr"/>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Additionsaufgaben halbschriftlich und schriftlich lösen.</t>
+          <t>Du benennst und bildest Verbformen in verschiedenen Zeiten (Präsens, Präteritum, Perfekt) richtig.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr"/>
@@ -890,18 +922,26 @@
       <c r="B38" s="2" t="inlineStr"/>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Subtraktionsaufgaben (-) mit und ohne Übergänge lösen.</t>
+          <t>Du kannst Wörter nach dem Alphabet sortieren und nachschlagen.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr"/>
-      <c r="B39" s="2" t="inlineStr"/>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Mathematik</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Zahl und Operation (Zahlenraum bis 1.000)</t>
+        </is>
+      </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Subtraktionsaufgaben mit Übertrag halbschriftlich und schriftlich lösen.</t>
+          <t>Du kannst dich im Zahlenraum bis 1000 orientieren.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr"/>
@@ -912,7 +952,7 @@
       <c r="B40" s="2" t="inlineStr"/>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Du löst die Multiplikationsaufgaben (*) des kleinen Einmaleins automatisiert.</t>
+          <t>Du kannst Additionsaufgaben (+) mit und ohne Übergänge lösen.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr"/>
@@ -923,7 +963,7 @@
       <c r="B41" s="2" t="inlineStr"/>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Du löst die Divisionsaufgaben (:) des kleinen Einmaleins automatisiert.</t>
+          <t>Du kannst Additionsaufgaben halbschriftlich und schriftlich lösen.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr"/>
@@ -934,7 +974,7 @@
       <c r="B42" s="2" t="inlineStr"/>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Divisionsaufgaben (:) mit Rest lösen.</t>
+          <t>Du kannst Subtraktionsaufgaben (-) mit und ohne Übergänge lösen.</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr"/>
@@ -945,7 +985,7 @@
       <c r="B43" s="2" t="inlineStr"/>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Du wählst geeignete Rechenstrategien aus und wendest sie an.</t>
+          <t>Du kannst Subtraktionsaufgaben mit Übertrag halbschriftlich und schriftlich lösen.</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr"/>
@@ -956,7 +996,7 @@
       <c r="B44" s="2" t="inlineStr"/>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Du nutzt geeignete Verfahren, um deine Ergebnisse zu überprüfen.</t>
+          <t>Du löst die Multiplikationsaufgaben (*) des kleinen Einmaleins automatisiert.</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr"/>
@@ -967,7 +1007,7 @@
       <c r="B45" s="2" t="inlineStr"/>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Sachaufgaben verstehen und eine passende Fragestellung entwickeln.</t>
+          <t>Du löst die Divisionsaufgaben (:) des kleinen Einmaleins automatisiert.</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr"/>
@@ -978,7 +1018,7 @@
       <c r="B46" s="2" t="inlineStr"/>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Du kannst zu Sachaufgaben Lösungswege finden und eine passende Antwort formulieren.</t>
+          <t>Du kannst Divisionsaufgaben (:) mit Rest lösen.</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr"/>
@@ -986,14 +1026,10 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr"/>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>Raum und Form</t>
-        </is>
-      </c>
+      <c r="B47" s="2" t="inlineStr"/>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Du kannst geometrischen Grundformen benennen und ihre besonderen Merkmale mit Fachbegriffen beschreiben.</t>
+          <t>Du wählst geeignete Rechenstrategien aus und wendest sie an.</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr"/>
@@ -1004,7 +1040,7 @@
       <c r="B48" s="2" t="inlineStr"/>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Du kannst geometrische Formen mit und ohne Lineal zeichnen.</t>
+          <t>Du nutzt geeignete Verfahren, um deine Ergebnisse zu überprüfen.</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr"/>
@@ -1015,7 +1051,7 @@
       <c r="B49" s="2" t="inlineStr"/>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Du vergrößerst oder verkleinerst Figuren nach Vorgaben.</t>
+          <t>Du kannst Sachaufgaben verstehen und eine passende Fragestellung entwickeln.</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr"/>
@@ -1026,7 +1062,7 @@
       <c r="B50" s="2" t="inlineStr"/>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Du erkennst komplexere geometrische Muster und kannst diese fortsetzen.</t>
+          <t>Du kannst zu Sachaufgaben Lösungswege finden und eine passende Antwort formulieren.</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr"/>
@@ -1034,10 +1070,14 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr"/>
-      <c r="B51" s="2" t="inlineStr"/>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Raum und Form</t>
+        </is>
+      </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Du kannst geometrische Körper benennen, mit Fachbegriffen beschreiben sie vergleichen und ihnen die entsprechenden Körpernetze zuordnen.</t>
+          <t>Du kannst geometrischen Grundformen benennen und ihre besonderen Merkmale mit Fachbegriffen beschreiben.</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr"/>
@@ -1048,7 +1088,7 @@
       <c r="B52" s="2" t="inlineStr"/>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Du überprüfst Figuren auf Achsensymmetrie und kannst zur Spiegelachse symmetrisch ergänzen.</t>
+          <t>Du kannst geometrische Formen mit und ohne Lineal zeichnen.</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr"/>
@@ -1059,7 +1099,7 @@
       <c r="B53" s="2" t="inlineStr"/>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Lagebeziehungen und Ansichten beschreiben.</t>
+          <t>Du vergrößerst oder verkleinerst Figuren nach Vorgaben.</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr"/>
@@ -1070,7 +1110,7 @@
       <c r="B54" s="2" t="inlineStr"/>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Lagepläne lesen und zeichnen sowie Wege auf Lageplänen finden, beschreiben und zeichnen.</t>
+          <t>Du erkennst komplexere geometrische Muster und kannst diese fortsetzen.</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr"/>
@@ -1078,14 +1118,10 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr"/>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>Größen und Messen</t>
-        </is>
-      </c>
+      <c r="B55" s="2" t="inlineStr"/>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Uhrzeiten sekundengenau ablesen, einstellen und notieren.</t>
+          <t>Du kannst geometrische Körper benennen, mit Fachbegriffen beschreiben sie vergleichen und ihnen die entsprechenden Körpernetze zuordnen.</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr"/>
@@ -1096,7 +1132,7 @@
       <c r="B56" s="2" t="inlineStr"/>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Zeitspannen bestimmen.</t>
+          <t>Du überprüfst Figuren auf Achsensymmetrie und kannst zur Spiegelachse symmetrisch ergänzen.</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr"/>
@@ -1107,7 +1143,7 @@
       <c r="B57" s="2" t="inlineStr"/>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Repräsentanten zu den Längeneinheiten mm, cm, m und km benennen und Längen abmessen.</t>
+          <t>Du kannst Lagebeziehungen und Ansichten beschreiben.</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr"/>
@@ -1118,7 +1154,7 @@
       <c r="B58" s="2" t="inlineStr"/>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Längenangaben in unterschiedlichen Schreibweisen darstellen.</t>
+          <t>Du kannst Lagepläne lesen und zeichnen sowie Wege auf Lageplänen finden, beschreiben und zeichnen.</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr"/>
@@ -1126,10 +1162,14 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr"/>
-      <c r="B59" s="2" t="inlineStr"/>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Größen und Messen</t>
+        </is>
+      </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Repräsentanten zu den Gewichtseinheiten g, kg und t benennen und Objekte wiegen.</t>
+          <t>Du kannst Uhrzeiten sekundengenau ablesen, einstellen und notieren.</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr"/>
@@ -1140,7 +1180,7 @@
       <c r="B60" s="2" t="inlineStr"/>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Gewichtsangaben in unterschiedlichen Schreibweisen darstellen.</t>
+          <t>Du kannst Zeitspannen bestimmen.</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr"/>
@@ -1151,7 +1191,7 @@
       <c r="B61" s="2" t="inlineStr"/>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Geldbeträge mit Scheinen und Münzen darstellen, miteinander vergleichen und ordnen.</t>
+          <t>Du kannst Repräsentanten zu den Längeneinheiten mm, cm, m und km benennen und Längen abmessen.</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr"/>
@@ -1162,7 +1202,7 @@
       <c r="B62" s="2" t="inlineStr"/>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Du kannst mit Geldbeträgen rechnen.</t>
+          <t>Du kannst Längenangaben in unterschiedlichen Schreibweisen darstellen.</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr"/>
@@ -1170,14 +1210,10 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr"/>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>Daten und Zufall</t>
-        </is>
-      </c>
+      <c r="B63" s="2" t="inlineStr"/>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Daten aus einer Tabelle oder einem Diagramm ablesen bzw. selbst erheben und in eine andere Darstellungsform übertragen.</t>
+          <t>Du kannst Repräsentanten zu den Gewichtseinheiten g, kg und t benennen und Objekte wiegen.</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr"/>
@@ -1188,7 +1224,7 @@
       <c r="B64" s="2" t="inlineStr"/>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Du kannst kombinatorische Aufgaben durch systematisches Vorgehen lösen und deine Lösung strategisch darstellen.</t>
+          <t>Du kannst Gewichtsangaben in unterschiedlichen Schreibweisen darstellen.</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr"/>
@@ -1199,7 +1235,7 @@
       <c r="B65" s="2" t="inlineStr"/>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Wahrscheinlichkeiten von einfachen Zufallsversuchen einschätzen, die Ergebnisse beschreiben und miteinander vergleichen.</t>
+          <t>Du kannst Geldbeträge mit Scheinen und Münzen darstellen, miteinander vergleichen und ordnen.</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr"/>
@@ -1207,14 +1243,10 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr"/>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>Problemlösen, Modellieren, Argumentieren, Darstellen/Kommunizieren</t>
-        </is>
-      </c>
+      <c r="B66" s="2" t="inlineStr"/>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Du stellst deine Ideen verständlich dar und kannst deinen Lösungsweg erklären sowie mit anderen vergleichen.</t>
+          <t>Du kannst mit Geldbeträgen rechnen.</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr"/>
@@ -1222,29 +1254,25 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr"/>
-      <c r="B67" s="2" t="inlineStr"/>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Daten und Zufall</t>
+        </is>
+      </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Begründungen und Argumente formulieren.</t>
+          <t>Du kannst Daten aus einer Tabelle oder einem Diagramm ablesen bzw. selbst erheben und in eine andere Darstellungsform übertragen.</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr"/>
       <c r="E67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>Sachunterricht</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>Erkenntnisgewinnung</t>
-        </is>
-      </c>
+      <c r="A68" s="2" t="inlineStr"/>
+      <c r="B68" s="2" t="inlineStr"/>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Du kannst zielführend Fragen stellen, um Wissen zu erwerben und Sachthemen zu verstehen.</t>
+          <t>Du kannst kombinatorische Aufgaben durch systematisches Vorgehen lösen und deine Lösung strategisch darstellen.</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr"/>
@@ -1255,7 +1283,7 @@
       <c r="B69" s="2" t="inlineStr"/>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Du kannst zu Sachthemen recherchieren, indem du verschiedene Quellen (Sachtexte, Interviews, Bild-, Text- und Sachquellen) auswertest.</t>
+          <t>Du kannst Wahrscheinlichkeiten von einfachen Zufallsversuchen einschätzen, die Ergebnisse beschreiben und miteinander vergleichen.</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr"/>
@@ -1263,10 +1291,14 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr"/>
-      <c r="B70" s="2" t="inlineStr"/>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Problemlösen, Modellieren, Argumentieren, Darstellen/Kommunizieren</t>
+        </is>
+      </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Du kannst einen Versuch (zum Pflanzenwachstum, zum Sprudelgas, zur magnetischen Wirkung von Strom) planen, aufbauen, durchführen und auswerten.</t>
+          <t>Du stellst deine Ideen verständlich dar und kannst deinen Lösungsweg erklären sowie mit anderen vergleichen.</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr"/>
@@ -1277,18 +1309,26 @@
       <c r="B71" s="2" t="inlineStr"/>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Daten zu (untersuchten Bereich einfügen) erheben, darstellen und auswerten.</t>
+          <t>Du kannst Begründungen und Argumente formulieren.</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr"/>
       <c r="E71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr"/>
-      <c r="B72" s="2" t="inlineStr"/>
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Sachunterricht</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Erkenntnisgewinnung</t>
+        </is>
+      </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Du kannst (Stadtpläne, Baupläne, mehrschrittige Anleitungen, PC-Programme, Apps) lesen und nutzen.</t>
+          <t>Du kannst zielführend Fragen stellen, um Wissen zu erwerben und Sachthemen zu verstehen.</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr"/>
@@ -1299,7 +1339,7 @@
       <c r="B73" s="2" t="inlineStr"/>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Du wendest Problemlösestrategien (im Klassenrat, bei Interessenskonflikten, bei technischen Fragestellungen) an.</t>
+          <t>Du kannst zu Sachthemen recherchieren, indem du verschiedene Quellen (Sachtexte, Interviews, Bild-, Text- und Sachquellen) auswertest.</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr"/>
@@ -1310,7 +1350,7 @@
       <c r="B74" s="2" t="inlineStr"/>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Du kannst (Modelle, technische Konstruktionen) (planen, bauen, erklären) und dadurch Erkenntnisse über (Fahrzeuge, Türme, Brücken, Pflanzen, Körperteile) gewinnen.</t>
+          <t>Du kannst einen Versuch (zum Pflanzenwachstum, zum Sprudelgas, zur magnetischen Wirkung von Strom) planen, aufbauen, durchführen und auswerten.</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr"/>
@@ -1318,14 +1358,10 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr"/>
-      <c r="B75" s="2" t="inlineStr">
-        <is>
-          <t>Kommunikation</t>
-        </is>
-      </c>
+      <c r="B75" s="2" t="inlineStr"/>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Du bringst dich in Unterrichtsgesprächen aktiv ein und zeigst dadurch dein Interesse an Sachthemen.</t>
+          <t>Du kannst Daten zu (untersuchten Bereich einfügen) erheben, darstellen und auswerten.</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr"/>
@@ -1336,7 +1372,7 @@
       <c r="B76" s="2" t="inlineStr"/>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Beobachtungen und Vermutungen von/ zu (Pflanzen, Tieren, Bildern, Gegenständen) äußern.</t>
+          <t>Du kannst (Stadtpläne, Baupläne, mehrschrittige Anleitungen, PC-Programme, Apps) lesen und nutzen.</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr"/>
@@ -1347,7 +1383,7 @@
       <c r="B77" s="2" t="inlineStr"/>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Du verwendest treffende Begriffe und sachlich angemessene Darstellungen (Symbole, Zeichnungen) zu den Sachthemen (Unterrichtsthemen einfügen).</t>
+          <t>Du wendest Problemlösestrategien (im Klassenrat, bei Interessenskonflikten, bei technischen Fragestellungen) an.</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr"/>
@@ -1358,7 +1394,7 @@
       <c r="B78" s="2" t="inlineStr"/>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Du nutzt geeignete Präsentations- und Darstellungsformen nach besprochenen Kriterien.</t>
+          <t>Du kannst (Modelle, technische Konstruktionen) (planen, bauen, erklären) und dadurch Erkenntnisse über (Fahrzeuge, Türme, Brücken, Pflanzen, Körperteile) gewinnen.</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr"/>
@@ -1368,12 +1404,12 @@
       <c r="A79" s="2" t="inlineStr"/>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Bewertung</t>
+          <t>Kommunikation</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Du kannst mit anderen darüber diskutieren, ob Dargestelltes real oder fiktiv ist.</t>
+          <t>Du bringst dich in Unterrichtsgesprächen aktiv ein und zeigst dadurch dein Interesse an Sachthemen.</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr"/>
@@ -1384,7 +1420,7 @@
       <c r="B80" s="2" t="inlineStr"/>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Du kannst (Ereignisse, Gegenstände) in der Zeit einordnen.</t>
+          <t>Du kannst Beobachtungen und Vermutungen von/ zu (Pflanzen, Tieren, Bildern, Gegenständen) äußern.</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr"/>
@@ -1395,7 +1431,7 @@
       <c r="B81" s="2" t="inlineStr"/>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Du benennst Maßnahmen zur Erhaltung der eigenen Gesundheit (Zähne/ gesunde Ernährung/ mein Körper).</t>
+          <t>Du verwendest treffende Begriffe und sachlich angemessene Darstellungen (Symbole, Zeichnungen) zu den Sachthemen (Unterrichtsthemen einfügen).</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr"/>
@@ -1406,7 +1442,7 @@
       <c r="B82" s="2" t="inlineStr"/>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Du kannst beschreiben, dass Umwelt und Natur im Sinne der Nachhaltigkeit geschützt werden müssen und gehst respektvoll mit Lebewesen um.</t>
+          <t>Du nutzt geeignete Präsentations- und Darstellungsformen nach besprochenen Kriterien.</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr"/>
@@ -1414,114 +1450,118 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr"/>
-      <c r="B83" s="2" t="inlineStr"/>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Bewertung</t>
+        </is>
+      </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Du kennst die Grundsätze des demokratischen Systems und wendest sie (im Klassenrat, bei Entscheidungsfindungen, politischen Diskussionen) an.</t>
+          <t>Du kannst mit anderen darüber diskutieren, ob Dargestelltes real oder fiktiv ist.</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr"/>
       <c r="E83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="inlineStr">
-        <is>
-          <t>Englisch</t>
-        </is>
-      </c>
+      <c r="A84" s="2" t="inlineStr"/>
       <c r="B84" s="2" t="inlineStr"/>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>(Kompetenzen hier ergänzen)</t>
+          <t>Du kannst (Ereignisse, Gegenstände) in der Zeit einordnen.</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr"/>
       <c r="E84" s="2" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>Sport</t>
-        </is>
-      </c>
+      <c r="A85" s="2" t="inlineStr"/>
       <c r="B85" s="2" t="inlineStr"/>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>(Kompetenzen hier ergänzen)</t>
+          <t>Du benennst Maßnahmen zur Erhaltung der eigenen Gesundheit (Zähne/ gesunde Ernährung/ mein Körper).</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr"/>
       <c r="E85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="inlineStr">
-        <is>
-          <t>Religion</t>
-        </is>
-      </c>
+      <c r="A86" s="2" t="inlineStr"/>
       <c r="B86" s="2" t="inlineStr"/>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>(Kompetenzen hier ergänzen)</t>
+          <t>Du kannst beschreiben, dass Umwelt und Natur im Sinne der Nachhaltigkeit geschützt werden müssen und gehst respektvoll mit Lebewesen um.</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr"/>
       <c r="E86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="inlineStr">
-        <is>
-          <t>Kunst</t>
-        </is>
-      </c>
+      <c r="A87" s="2" t="inlineStr"/>
       <c r="B87" s="2" t="inlineStr"/>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Du beteiligst dich an Unterrichtsgesprächen und zeigst so Interesse an künstlerischen Themen.</t>
+          <t>Du kennst die Grundsätze des demokratischen Systems und wendest sie (im Klassenrat, bei Entscheidungsfindungen, politischen Diskussionen) an.</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr"/>
       <c r="E87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="inlineStr"/>
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Englisch</t>
+        </is>
+      </c>
       <c r="B88" s="2" t="inlineStr"/>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Du nutzt Buntstifte, Wasserfarben, Acrylfarben und selbst ausgewählte Bastelmaterialien für deine Werke.</t>
+          <t>(Kompetenzen hier ergänzen)</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr"/>
       <c r="E88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="inlineStr"/>
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
       <c r="B89" s="2" t="inlineStr"/>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Du beachtest gestalterische Kriterien bei der Umsetzung eines Themas.</t>
+          <t>(Kompetenzen hier ergänzen)</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr"/>
       <c r="E89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="inlineStr"/>
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
       <c r="B90" s="2" t="inlineStr"/>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Du hast eigene Ideen zur Gestaltung.</t>
+          <t>(Kompetenzen hier ergänzen)</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr"/>
       <c r="E90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="inlineStr"/>
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Kunst</t>
+        </is>
+      </c>
       <c r="B91" s="2" t="inlineStr"/>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Du setzt deine Ideen selbstständig um.</t>
+          <t>Du beteiligst dich an Unterrichtsgesprächen und zeigst so Interesse an künstlerischen Themen.</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr"/>
@@ -1532,7 +1572,7 @@
       <c r="B92" s="2" t="inlineStr"/>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Du stellst deine Werke in der vorgesehenen Zeit sinnvoll fertig.</t>
+          <t>Du nutzt Buntstifte, Wasserfarben, Acrylfarben und selbst ausgewählte Bastelmaterialien für deine Werke.</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr"/>
@@ -1543,7 +1583,7 @@
       <c r="B93" s="2" t="inlineStr"/>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Tipps annehmen und sinnvoll für die eigene Arbeit nutzen.</t>
+          <t>Du beachtest gestalterische Kriterien bei der Umsetzung eines Themas.</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr"/>
@@ -1554,7 +1594,7 @@
       <c r="B94" s="2" t="inlineStr"/>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Du kannst deine eigenen Kunstwerke und die anderer Künstler beschreiben.</t>
+          <t>Du hast eigene Ideen zur Gestaltung.</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr"/>
@@ -1565,7 +1605,7 @@
       <c r="B95" s="2" t="inlineStr"/>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Du begründest deine Meinung zu Kunstwerken.</t>
+          <t>Du setzt deine Ideen selbstständig um.</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr"/>
@@ -1576,7 +1616,7 @@
       <c r="B96" s="2" t="inlineStr"/>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Du kennst Fachbegriffe und nutzt sie passend.</t>
+          <t>Du stellst deine Werke in der vorgesehenen Zeit sinnvoll fertig.</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr"/>
@@ -1587,22 +1627,18 @@
       <c r="B97" s="2" t="inlineStr"/>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Du kannst ausdrücken, ob du dich an die Gestaltungsvorgaben gehalten hast.</t>
+          <t>Du kannst Tipps annehmen und sinnvoll für die eigene Arbeit nutzen.</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr"/>
       <c r="E97" s="2" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="inlineStr">
-        <is>
-          <t>Musik</t>
-        </is>
-      </c>
+      <c r="A98" s="2" t="inlineStr"/>
       <c r="B98" s="2" t="inlineStr"/>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Du beteiligst dich interessiert an den musikalischen Aktivitäten.</t>
+          <t>Du kannst deine eigenen Kunstwerke und die anderer Künstler beschreiben.</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr"/>
@@ -1613,7 +1649,7 @@
       <c r="B99" s="2" t="inlineStr"/>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Du beteiligst dich aktiv an Unterrichtsgesprächen.</t>
+          <t>Du begründest deine Meinung zu Kunstwerken.</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr"/>
@@ -1624,7 +1660,7 @@
       <c r="B100" s="2" t="inlineStr"/>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Du findest passende Bewegungen und entwickelst Choreografien zu unterschiedlicher Musik.</t>
+          <t>Du kennst Fachbegriffe und nutzt sie passend.</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr"/>
@@ -1635,18 +1671,22 @@
       <c r="B101" s="2" t="inlineStr"/>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Rhythmen umsetzen.</t>
+          <t>Du kannst ausdrücken, ob du dich an die Gestaltungsvorgaben gehalten hast.</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr"/>
       <c r="E101" s="2" t="inlineStr"/>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="inlineStr"/>
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Musik</t>
+        </is>
+      </c>
       <c r="B102" s="2" t="inlineStr"/>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Du singst unsere Lieder mit.</t>
+          <t>Du beteiligst dich interessiert an den musikalischen Aktivitäten.</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr"/>
@@ -1657,7 +1697,7 @@
       <c r="B103" s="2" t="inlineStr"/>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Du tanzt vorgegebene Tänze nach.</t>
+          <t>Du beteiligst dich aktiv an Unterrichtsgesprächen.</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr"/>
@@ -1668,7 +1708,7 @@
       <c r="B104" s="2" t="inlineStr"/>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Du kennst alle Orff-Instrumente und spielst sie rhythmisch und technisch korrekt.</t>
+          <t>Du findest passende Bewegungen und entwickelst Choreografien zu unterschiedlicher Musik.</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr"/>
@@ -1679,7 +1719,7 @@
       <c r="B105" s="2" t="inlineStr"/>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Du kennst Orchester-Instrumente.</t>
+          <t>Du kannst Rhythmen umsetzen.</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr"/>
@@ -1690,7 +1730,7 @@
       <c r="B106" s="2" t="inlineStr"/>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Du kennst musikalische Gestaltungsmittel wie hoch-tief, laut-leise, schnell-langsam, traurig-fröhlich und kannst sie umsetzen.</t>
+          <t>Du singst unsere Lieder mit.</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr"/>
@@ -1701,7 +1741,7 @@
       <c r="B107" s="2" t="inlineStr"/>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Du kannst Notenwerte benennen und umsetzen.</t>
+          <t>Du tanzt vorgegebene Tänze nach.</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr"/>
@@ -1712,11 +1752,55 @@
       <c r="B108" s="2" t="inlineStr"/>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Du nutzt musikalische Fachbegriffe.</t>
+          <t>Du kennst alle Orff-Instrumente und spielst sie rhythmisch und technisch korrekt.</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr"/>
       <c r="E108" s="2" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr"/>
+      <c r="B109" s="2" t="inlineStr"/>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>Du kennst Orchester-Instrumente.</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr"/>
+      <c r="E109" s="2" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr"/>
+      <c r="B110" s="2" t="inlineStr"/>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Du kennst musikalische Gestaltungsmittel wie hoch-tief, laut-leise, schnell-langsam, traurig-fröhlich und kannst sie umsetzen.</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr"/>
+      <c r="E110" s="2" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr"/>
+      <c r="B111" s="2" t="inlineStr"/>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Du kannst Notenwerte benennen und umsetzen.</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr"/>
+      <c r="E111" s="2" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr"/>
+      <c r="B112" s="2" t="inlineStr"/>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>Du nutzt musikalische Fachbegriffe.</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr"/>
+      <c r="E112" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>